<commit_message>
update tableau de compétences
</commit_message>
<xml_diff>
--- a/public/files/Tableau de compétences.xlsx
+++ b/public/files/Tableau de compétences.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t xml:space="preserve">BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -122,31 +122,44 @@
     <t xml:space="preserve">WorkTogether</t>
   </si>
   <si>
+    <t xml:space="preserve">18/11/2024 au 24/03/2025</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
   </si>
   <si>
     <t xml:space="preserve">Portfolio</t>
   </si>
   <si>
+    <t xml:space="preserve">11/01/2025 au 24/03/2024</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
     <t xml:space="preserve">Site vitrine RPE Val d’izé</t>
   </si>
   <si>
+    <t xml:space="preserve">08/05/2024 au 07/06/2024</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
     <t xml:space="preserve">Projet de tests d’application mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15/01/2025 au 28/02/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* \-??\ [$€-1]_-"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -550,7 +563,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -631,16 +644,20 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -936,7 +953,7 @@
   <sheetFormatPr defaultColWidth="10.84765625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="70.42"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="18.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="9" style="2" width="11.43"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="44" style="1" width="10.85"/>
@@ -1079,37 +1096,41 @@
       <c r="A9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="20"/>
+      <c r="B9" s="20" t="s">
+        <v>26</v>
+      </c>
       <c r="C9" s="21"/>
       <c r="D9" s="21"/>
       <c r="E9" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="22"/>
     </row>
     <row r="10" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="20"/>
+        <v>28</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>29</v>
+      </c>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
       <c r="E10" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
       <c r="H10" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19"/>
-      <c r="B11" s="20"/>
+      <c r="B11" s="23"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
@@ -1119,7 +1140,7 @@
     </row>
     <row r="12" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19"/>
-      <c r="B12" s="20"/>
+      <c r="B12" s="23"/>
       <c r="C12" s="21"/>
       <c r="D12" s="21"/>
       <c r="E12" s="21"/>
@@ -1129,7 +1150,7 @@
     </row>
     <row r="13" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="19"/>
-      <c r="B13" s="20"/>
+      <c r="B13" s="23"/>
       <c r="C13" s="21"/>
       <c r="D13" s="21"/>
       <c r="E13" s="21"/>
@@ -1139,7 +1160,7 @@
     </row>
     <row r="14" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
+      <c r="B14" s="23"/>
       <c r="C14" s="21"/>
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
@@ -1149,7 +1170,7 @@
     </row>
     <row r="15" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="19"/>
-      <c r="B15" s="20"/>
+      <c r="B15" s="23"/>
       <c r="C15" s="21"/>
       <c r="D15" s="21"/>
       <c r="E15" s="21"/>
@@ -1159,7 +1180,7 @@
     </row>
     <row r="16" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="19"/>
-      <c r="B16" s="20"/>
+      <c r="B16" s="23"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
@@ -1169,7 +1190,7 @@
     </row>
     <row r="17" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19"/>
-      <c r="B17" s="20"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="21"/>
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
@@ -1179,7 +1200,7 @@
     </row>
     <row r="18" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="19"/>
-      <c r="B18" s="20"/>
+      <c r="B18" s="23"/>
       <c r="C18" s="21"/>
       <c r="D18" s="21"/>
       <c r="E18" s="21"/>
@@ -1188,38 +1209,40 @@
       <c r="H18" s="22"/>
     </row>
     <row r="19" s="17" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
+      <c r="A19" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
     </row>
     <row r="20" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="20"/>
-      <c r="C20" s="24"/>
+        <v>31</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="25"/>
       <c r="D20" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F20" s="21"/>
       <c r="G20" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H20" s="22"/>
     </row>
     <row r="21" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="19"/>
-      <c r="B21" s="20"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
@@ -1229,7 +1252,7 @@
     </row>
     <row r="22" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19"/>
-      <c r="B22" s="20"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="21"/>
       <c r="D22" s="21"/>
       <c r="E22" s="21"/>
@@ -1239,7 +1262,7 @@
     </row>
     <row r="23" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="19"/>
-      <c r="B23" s="20"/>
+      <c r="B23" s="23"/>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
       <c r="E23" s="21"/>
@@ -1249,7 +1272,7 @@
     </row>
     <row r="24" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="19"/>
-      <c r="B24" s="20"/>
+      <c r="B24" s="23"/>
       <c r="C24" s="21"/>
       <c r="D24" s="21"/>
       <c r="E24" s="21"/>
@@ -1259,7 +1282,7 @@
     </row>
     <row r="25" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
+      <c r="B25" s="23"/>
       <c r="C25" s="21"/>
       <c r="D25" s="21"/>
       <c r="E25" s="21"/>
@@ -1269,7 +1292,7 @@
     </row>
     <row r="26" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="19"/>
-      <c r="B26" s="20"/>
+      <c r="B26" s="23"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
@@ -1278,34 +1301,36 @@
       <c r="H26" s="22"/>
     </row>
     <row r="27" s="17" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
+      <c r="A27" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
     </row>
     <row r="28" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="20"/>
+        <v>34</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>35</v>
+      </c>
       <c r="C28" s="21"/>
       <c r="D28" s="21"/>
       <c r="E28" s="21"/>
       <c r="F28" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G28" s="21"/>
       <c r="H28" s="22"/>
     </row>
     <row r="29" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19"/>
-      <c r="B29" s="20"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="21"/>
       <c r="D29" s="21"/>
       <c r="E29" s="21"/>
@@ -1315,7 +1340,7 @@
     </row>
     <row r="30" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19"/>
-      <c r="B30" s="20"/>
+      <c r="B30" s="23"/>
       <c r="C30" s="21"/>
       <c r="D30" s="21"/>
       <c r="E30" s="21"/>
@@ -1325,7 +1350,7 @@
     </row>
     <row r="31" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="19"/>
-      <c r="B31" s="20"/>
+      <c r="B31" s="23"/>
       <c r="C31" s="21"/>
       <c r="D31" s="21"/>
       <c r="E31" s="21"/>
@@ -1335,7 +1360,7 @@
     </row>
     <row r="32" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="19"/>
-      <c r="B32" s="20"/>
+      <c r="B32" s="23"/>
       <c r="C32" s="21"/>
       <c r="D32" s="21"/>
       <c r="E32" s="21"/>
@@ -1344,8 +1369,8 @@
       <c r="H32" s="22"/>
     </row>
     <row r="33" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25"/>
-      <c r="B33" s="20"/>
+      <c r="A33" s="26"/>
+      <c r="B33" s="23"/>
       <c r="C33" s="21"/>
       <c r="D33" s="21"/>
       <c r="E33" s="21"/>
@@ -1354,24 +1379,24 @@
       <c r="H33" s="22"/>
     </row>
     <row r="34" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="26"/>
-      <c r="B34" s="27"/>
-      <c r="C34" s="28"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="28"/>
-      <c r="F34" s="28"/>
-      <c r="G34" s="28"/>
-      <c r="H34" s="29"/>
+      <c r="A34" s="27"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="30"/>
     </row>
     <row r="35" s="17" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="30"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
+      <c r="A35" s="31"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
     </row>
     <row r="36" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="37" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>